<commit_message>
changed trades in strategy to a pd.df - started implementing StrategyAnalysis
</commit_message>
<xml_diff>
--- a/stockMarket/technicalAnalysis/templates/template.xlsx
+++ b/stockMarket/technicalAnalysis/templates/template.xlsx
@@ -5,13 +5,13 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="overview" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="analytics" sheetId="2" state="visible" r:id="rId4"/>
-    <sheet name="analytics_all_trades" sheetId="3" state="visible" r:id="rId5"/>
-    <sheet name="stocks" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="overview" sheetId="1" state="visible" r:id="rId2"/>
+    <sheet name="analytics" sheetId="2" state="visible" r:id="rId3"/>
+    <sheet name="analytics_all_trades" sheetId="3" state="visible" r:id="rId4"/>
+    <sheet name="stocks" sheetId="4" state="visible" r:id="rId5"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -484,7 +484,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="4" fillId="4" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="4" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -704,121 +704,15 @@
 </styleSheet>
 </file>
 
-<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office">
-  <a:themeElements>
-    <a:clrScheme name="LibreOffice">
-      <a:dk1>
-        <a:srgbClr val="000000"/>
-      </a:dk1>
-      <a:lt1>
-        <a:srgbClr val="ffffff"/>
-      </a:lt1>
-      <a:dk2>
-        <a:srgbClr val="000000"/>
-      </a:dk2>
-      <a:lt2>
-        <a:srgbClr val="ffffff"/>
-      </a:lt2>
-      <a:accent1>
-        <a:srgbClr val="18a303"/>
-      </a:accent1>
-      <a:accent2>
-        <a:srgbClr val="0369a3"/>
-      </a:accent2>
-      <a:accent3>
-        <a:srgbClr val="a33e03"/>
-      </a:accent3>
-      <a:accent4>
-        <a:srgbClr val="8e03a3"/>
-      </a:accent4>
-      <a:accent5>
-        <a:srgbClr val="c99c00"/>
-      </a:accent5>
-      <a:accent6>
-        <a:srgbClr val="c9211e"/>
-      </a:accent6>
-      <a:hlink>
-        <a:srgbClr val="0000ee"/>
-      </a:hlink>
-      <a:folHlink>
-        <a:srgbClr val="551a8b"/>
-      </a:folHlink>
-    </a:clrScheme>
-    <a:fontScheme name="Office">
-      <a:majorFont>
-        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
-        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
-        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
-      </a:majorFont>
-      <a:minorFont>
-        <a:latin typeface="Arial" pitchFamily="0" charset="1"/>
-        <a:ea typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
-        <a:cs typeface="DejaVu Sans" pitchFamily="0" charset="1"/>
-      </a:minorFont>
-    </a:fontScheme>
-    <a:fmtScheme>
-      <a:fillStyleLst>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-      </a:fillStyleLst>
-      <a:lnStyleLst>
-        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
-          <a:prstDash val="solid"/>
-          <a:miter/>
-        </a:ln>
-        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
-          <a:prstDash val="solid"/>
-          <a:miter/>
-        </a:ln>
-        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
-          <a:prstDash val="solid"/>
-          <a:miter/>
-        </a:ln>
-      </a:lnStyleLst>
-      <a:effectStyleLst>
-        <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-      </a:effectStyleLst>
-      <a:bgFillStyleLst>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr"/>
-        </a:solidFill>
-      </a:bgFillStyleLst>
-    </a:fmtScheme>
-  </a:themeElements>
-</a:theme>
-</file>
-
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:L1000"/>
-  <sheetFormatPr defaultColWidth="12.65234375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.66796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="19.76"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="19.77"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="12.75"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="10.25"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="11.38"/>
@@ -1034,10 +928,7 @@
       <c r="H14" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="I14" s="22" t="n">
-        <f aca="false">COUNTIF(analytics!J:J,"W")</f>
-        <v>0</v>
-      </c>
+      <c r="I14" s="22"/>
       <c r="J14" s="3"/>
       <c r="K14" s="3"/>
       <c r="L14" s="3"/>
@@ -1046,10 +937,7 @@
       <c r="H15" s="21" t="s">
         <v>15</v>
       </c>
-      <c r="I15" s="22" t="n">
-        <f aca="false">COUNTIF(analytics!J:J,"L")</f>
-        <v>0</v>
-      </c>
+      <c r="I15" s="22"/>
       <c r="J15" s="3"/>
       <c r="K15" s="3"/>
       <c r="L15" s="3"/>
@@ -1058,10 +946,7 @@
       <c r="H16" s="21" t="s">
         <v>16</v>
       </c>
-      <c r="I16" s="23" t="e">
-        <f aca="false">I14/I15</f>
-        <v>#DIV/0!</v>
-      </c>
+      <c r="I16" s="23"/>
       <c r="J16" s="3"/>
       <c r="K16" s="3"/>
       <c r="L16" s="3"/>
@@ -1070,10 +955,7 @@
       <c r="H17" s="21" t="s">
         <v>17</v>
       </c>
-      <c r="I17" s="23" t="e">
-        <f aca="false">I14/(I14+I15)</f>
-        <v>#DIV/0!</v>
-      </c>
+      <c r="I17" s="23"/>
       <c r="J17" s="3"/>
       <c r="K17" s="3"/>
       <c r="L17" s="3"/>
@@ -1082,10 +964,7 @@
       <c r="H18" s="21" t="s">
         <v>18</v>
       </c>
-      <c r="I18" s="24" t="e">
-        <f aca="false">AVERAGE(analytics!H:H)</f>
-        <v>#DIV/0!</v>
-      </c>
+      <c r="I18" s="24"/>
       <c r="J18" s="3"/>
       <c r="K18" s="3"/>
       <c r="L18" s="3"/>
@@ -1094,10 +973,7 @@
       <c r="H19" s="21" t="s">
         <v>19</v>
       </c>
-      <c r="I19" s="24" t="e">
-        <f aca="false">AVERAGE(analytics!I:I)</f>
-        <v>#DIV/0!</v>
-      </c>
+      <c r="I19" s="24"/>
       <c r="J19" s="3"/>
       <c r="K19" s="3"/>
       <c r="L19" s="3"/>
@@ -1113,9 +989,9 @@
       <c r="H21" s="26" t="s">
         <v>20</v>
       </c>
-      <c r="I21" s="27" t="e">
+      <c r="I21" s="27" t="n">
         <f aca="false">(1 + I18)*$I$17-1</f>
-        <v>#DIV/0!</v>
+        <v>-1</v>
       </c>
       <c r="J21" s="3"/>
       <c r="K21" s="3"/>
@@ -1125,9 +1001,9 @@
       <c r="H22" s="26" t="s">
         <v>21</v>
       </c>
-      <c r="I22" s="27" t="e">
+      <c r="I22" s="27" t="n">
         <f aca="false">(1 + I19)*$I$17-1</f>
-        <v>#DIV/0!</v>
+        <v>-1</v>
       </c>
       <c r="J22" s="3"/>
       <c r="K22" s="3"/>
@@ -8002,8 +7878,8 @@
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageSetup paperSize="1" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -8012,18 +7888,18 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AG1000"/>
-  <sheetFormatPr defaultColWidth="11.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="7.27"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="10.76"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="10.77"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="15.48"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="31" width="23.07"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="7.42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="31" width="23.08"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="7.41"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="12.15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="31" width="23.5"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="4.63"/>
@@ -8032,8 +7908,8 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="13.95"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="20.77"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="11.58"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="16.88"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="19.11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="16.87"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="19.12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="9.92"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="1" width="11.45"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="1" width="16.6"/>
@@ -28110,8 +27986,8 @@
     <mergeCell ref="Y1:AE1"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageSetup paperSize="1" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -28120,18 +27996,18 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AG1000"/>
-  <sheetFormatPr defaultColWidth="11.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="7.27"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="10.76"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="10.77"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="15.48"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="31" width="23.07"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="7.42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="31" width="23.08"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="7.41"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="12.15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="31" width="23.5"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="4.63"/>
@@ -28140,8 +28016,8 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="13.95"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="20.77"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="11.58"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="16.88"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="19.11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="16.87"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="19.12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="9.92"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="1" width="11.45"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="1" width="16.6"/>
@@ -48218,8 +48094,8 @@
     <mergeCell ref="Y1:AE1"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageSetup paperSize="1" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -48228,23 +48104,23 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:N1000"/>
-  <sheetFormatPr defaultColWidth="12.65234375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.66796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="13.4"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="11.31"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="7.27"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="1" width="11.72"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="10.76"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="10.77"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="12.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="7.42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="7.41"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="9.92"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="5.06"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="7.42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="7.41"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="17.29"/>
   </cols>
   <sheetData>
@@ -61294,8 +61170,8 @@
     <mergeCell ref="I1:L1"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageSetup paperSize="1" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>

</xml_diff>